<commit_message>
Retraites : calage sur l'IPP (note n° 129), onglet Abattement de 10 % et comparaison à rendement égal
- CSG des retraités : options « taux normal » et « taux médian et normal » (taux réduit épargné), assiettes calées
  sur l'IPP (1,5 et 4,2 Md€ nets), recette nette reversée aux actifs ; nuance sur le profil en U.
- Gel : distribution des pensions portée à 2027 (médiane 1 639 €) et part de base décroissante avec la pension,
  calées sur les quatre chiffrages de l'IPP ; revalorisation 2027 de 2,5 % par défaut ; gain net reversé.
- Nouvel onglet Abattement de 10 % (suppression ou plafond abaissé), hausse d'impôt d'un foyer.
- Encadré « trois pistes, un même rendement » en tête de Simuler ; tableau des neuf scénarios et calage dans Méthode.
- Santé, classeurs Excel et tests mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188qNw1StBQkFA1rFcQwdyx
</commit_message>
<xml_diff>
--- a/site/chiffrages/Chiffrage_Sante.xlsx
+++ b/site/chiffrages/Chiffrage_Sante.xlsx
@@ -1288,7 +1288,7 @@
         <v>31</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>225</v>
+        <v>190.5</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>32</v>
@@ -1299,7 +1299,7 @@
         <v>33</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>87</v>
+        <v>118.7</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>34</v>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B25" s="16" t="n">
         <f aca="false">IF(Leviers!$B$4="Oui",Leviers!$B$14*(Leviers!$B$12-Leviers!$B$13),0)</f>
-        <v>2.025</v>
+        <v>1.7145</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B26" s="16" t="n">
         <f aca="false">Leviers!$B$5*(Leviers!$B$15+Leviers!$B$14)*Leviers!$B$16</f>
-        <v>2.0904</v>
+        <v>2.07164</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B27" s="17" t="n">
         <f aca="false">B25+B26</f>
-        <v>4.1154</v>
+        <v>3.78614</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B29" s="17" t="n">
         <f aca="false">B27-B28</f>
-        <v>0.750369469403287</v>
+        <v>0.421109469403286</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B30" s="19" t="n">
         <f aca="false">IF(B29&gt;0,B29/ABS(Leviers!$B$21),0)</f>
-        <v>0.0543745992321222</v>
+        <v>0.0305151789422671</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="B35" s="17" t="n">
         <f aca="false">B27-B28*B32</f>
-        <v>1.52523936308814</v>
+        <v>1.19597936308814</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Retraites : calage sur l'IPP (note n° 129), onglet Abattement de 10 % et comparaison à rendement égal (#17)
- CSG des retraités : options « taux normal » et « taux médian et normal » (taux réduit épargné), assiettes calées
  sur l'IPP (1,5 et 4,2 Md€ nets), recette nette reversée aux actifs ; nuance sur le profil en U.
- Gel : distribution des pensions portée à 2027 (médiane 1 639 €) et part de base décroissante avec la pension,
  calées sur les quatre chiffrages de l'IPP ; revalorisation 2027 de 2,5 % par défaut ; gain net reversé.
- Nouvel onglet Abattement de 10 % (suppression ou plafond abaissé), hausse d'impôt d'un foyer.
- Encadré « trois pistes, un même rendement » en tête de Simuler ; tableau des neuf scénarios et calage dans Méthode.
- Santé, classeurs Excel et tests mis à jour.


Claude-Session: https://claude.ai/code/session_0188qNw1StBQkFA1rFcQwdyx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/chiffrages/Chiffrage_Sante.xlsx
+++ b/site/chiffrages/Chiffrage_Sante.xlsx
@@ -1288,7 +1288,7 @@
         <v>31</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>225</v>
+        <v>190.5</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>32</v>
@@ -1299,7 +1299,7 @@
         <v>33</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>87</v>
+        <v>118.7</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>34</v>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B25" s="16" t="n">
         <f aca="false">IF(Leviers!$B$4="Oui",Leviers!$B$14*(Leviers!$B$12-Leviers!$B$13),0)</f>
-        <v>2.025</v>
+        <v>1.7145</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B26" s="16" t="n">
         <f aca="false">Leviers!$B$5*(Leviers!$B$15+Leviers!$B$14)*Leviers!$B$16</f>
-        <v>2.0904</v>
+        <v>2.07164</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B27" s="17" t="n">
         <f aca="false">B25+B26</f>
-        <v>4.1154</v>
+        <v>3.78614</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B29" s="17" t="n">
         <f aca="false">B27-B28</f>
-        <v>0.750369469403287</v>
+        <v>0.421109469403286</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B30" s="19" t="n">
         <f aca="false">IF(B29&gt;0,B29/ABS(Leviers!$B$21),0)</f>
-        <v>0.0543745992321222</v>
+        <v>0.0305151789422671</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="B35" s="17" t="n">
         <f aca="false">B27-B28*B32</f>
-        <v>1.52523936308814</v>
+        <v>1.19597936308814</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>